<commit_message>
Added External service support and TCP/IP services
</commit_message>
<xml_diff>
--- a/schema/ADRM/Business Rules.xlsx
+++ b/schema/ADRM/Business Rules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/82cfe7acc6d68563/Documents/github/HL7-Validator/schema/ADRM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="8_{D9E72346-FD95-4C6F-AFA1-43E83E9B8086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{797F5AC8-7471-4920-BC94-79A600B751EF}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{D9E72346-FD95-4C6F-AFA1-43E83E9B8086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B03E1C42-0AD4-40B3-8630-EEE417AC8CB4}"/>
   <bookViews>
-    <workbookView xWindow="22290" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22290" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datatype rules" sheetId="4" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="segment rules" sheetId="2" r:id="rId3"/>
     <sheet name="XPath rules" sheetId="3" r:id="rId4"/>
     <sheet name="parser rules" sheetId="5" r:id="rId5"/>
+    <sheet name="external rules" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="194">
   <si>
     <t>rule</t>
   </si>
@@ -186,24 +187,12 @@
     <t>HL7 Version and Internationalization</t>
   </si>
   <si>
-    <t>HL7au:000040.3</t>
-  </si>
-  <si>
     <t>HL7au:000040.4</t>
   </si>
   <si>
-    <t>HL7 Internal Version Lab</t>
-  </si>
-  <si>
-    <t>HL7 Internal Version Referral</t>
-  </si>
-  <si>
     <t>ORM_O01,ORU_R01</t>
   </si>
   <si>
-    <t>REF_I12,RRI_I12</t>
-  </si>
-  <si>
     <t>MSH-17</t>
   </si>
   <si>
@@ -585,12 +574,6 @@
     <t>wellFormed,noNesting,noOLE,noEmbeddedFonts</t>
   </si>
   <si>
-    <t>/REF_I12[MSH.12/VID/text() = "HL7AU-OO-REF-SIMPLIFIED_201706-L1"]</t>
-  </si>
-  <si>
-    <t>/ORU_R01[MSH.12/VID/text() = "HL7AU-OO-REF-SIMPLIFIED_201706-L1"]</t>
-  </si>
-  <si>
     <t>//ORU_R01.OBSERVATION/OBX/OBX.6/CE.1[../CE.3/text() = "UCUM"]</t>
   </si>
   <si>
@@ -607,13 +590,46 @@
   </si>
   <si>
     <t>//ORU_R01.RESULT/OBX/OBX.5/ED.5[../../OBX.2/text() = "ED" and ../../OBX.1/CE.1/text() = "RTF" and ../../OBX.1/CE.3/text() = "AUSPDI" and ../ED.2[text() = "TX"] and ../ED.3[text() = "RTF"] and ../ED.4[text() = "A"]]</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>APIkey</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>csiroUCUM</t>
+  </si>
+  <si>
+    <t>https://tx.ontoserver.csiro.au/fhir/CodeSystem/$validate-code</t>
+  </si>
+  <si>
+    <t>ORM_O01,ORU_R01,REF_I12,RRI_I12</t>
+  </si>
+  <si>
+    <t>HL7 Internal Version</t>
+  </si>
+  <si>
+    <t>//ORU_R01[MSH.12/VID/text() = "HL7AU-OO-REF-SIMPLIFIED_201706-L1"]</t>
+  </si>
+  <si>
+    <t>//REF_I12[MSH.12/VID/text() = "HL7AU-OO-REF-SIMPLIFIED_201706-L1"]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -626,6 +642,14 @@
       <color rgb="FF292A2E"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -651,10 +675,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -662,8 +687,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -958,13 +985,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
         <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -975,254 +1002,254 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
         <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E11" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
         <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
         <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
       </c>
       <c r="D15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
         <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E17" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E18" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1232,7 +1259,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="67.3984375" bestFit="1" customWidth="1"/>
@@ -1245,7 +1272,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
         <v>20</v>
@@ -1356,7 +1383,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -1367,36 +1394,36 @@
     </row>
     <row r="8" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B8" t="s">
         <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
         <v>45</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D9" t="s">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
@@ -1421,7 +1448,7 @@
         <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>190</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>48</v>
@@ -1430,89 +1457,72 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>44</v>
-      </c>
       <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>118</v>
       </c>
       <c r="D12" t="s">
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
         <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D13" t="s">
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>76</v>
+      </c>
+      <c r="B15" t="s">
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D15" t="s">
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>80</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" t="s">
-        <v>125</v>
-      </c>
-      <c r="D16" t="s">
-        <v>4</v>
-      </c>
-      <c r="F16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1559,13 +1569,13 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E2" t="s">
         <v>36</v>
@@ -1585,10 +1595,10 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E3" t="s">
         <v>36</v>
@@ -1605,13 +1615,13 @@
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G4" t="s">
         <v>42</v>
@@ -1622,13 +1632,13 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="G5" t="s">
         <v>43</v>
@@ -1636,53 +1646,53 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
         <v>36</v>
@@ -1691,44 +1701,44 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D9" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E10" t="s">
         <v>36</v>
@@ -1737,7 +1747,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
@@ -1745,16 +1755,16 @@
         <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C11" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D11" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G11" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
@@ -1762,16 +1772,16 @@
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
@@ -1779,16 +1789,16 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1861,13 +1871,13 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F2" t="s">
         <v>36</v>
@@ -1876,38 +1886,38 @@
         <v>1</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="E3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="E4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F4" t="s">
         <v>36</v>
@@ -1916,44 +1926,44 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="E5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="H6" t="s">
         <v>38</v>
@@ -1962,58 +1972,58 @@
         <v>39</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="50.35" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H7" t="s">
         <v>38</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H8" t="s">
         <v>38</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F9" t="s">
         <v>36</v>
@@ -2025,10 +2035,10 @@
         <v>38</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2053,13 +2063,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E1" t="s">
         <v>7</v>
@@ -2067,174 +2077,233 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" t="s">
         <v>167</v>
       </c>
-      <c r="C4" t="s">
-        <v>171</v>
-      </c>
       <c r="E4" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E5" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E6" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C7" t="s">
         <v>167</v>
       </c>
-      <c r="C7" t="s">
-        <v>171</v>
-      </c>
       <c r="D7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E7" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E8" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E9" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E10" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C11" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D11" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E11" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C12" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E12" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB807017-95D5-46C6-8199-291D5344FE3E}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="5.9296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="58.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{46D6215E-12D0-4901-8694-94E01854CE92}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>